<commit_message>
[v0.19] 股指信号调整 09-16=0.5(仓位15%) 09-17=0.3(待生效) 净值2.6054
</commit_message>
<xml_diff>
--- a/数据/原始数据/股指期货信号.xlsx
+++ b/数据/原始数据/股指期货信号.xlsx
@@ -78,7 +78,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -94,6 +94,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -471,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2215"/>
+  <dimension ref="A1:B2217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="18.5" customWidth="1" style="1" min="1" max="1"/>
@@ -17651,7 +17652,7 @@
       <c r="A2202" s="1" t="n">
         <v>46262</v>
       </c>
-      <c r="B2202" t="n">
+      <c r="B2202" s="0" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -17659,7 +17660,7 @@
       <c r="A2203" s="1" t="n">
         <v>46263</v>
       </c>
-      <c r="B2203" t="n">
+      <c r="B2203" s="0" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -17667,7 +17668,7 @@
       <c r="A2204" s="1" t="n">
         <v>46264</v>
       </c>
-      <c r="B2204" t="n">
+      <c r="B2204" s="0" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -17675,7 +17676,7 @@
       <c r="A2205" s="1" t="n">
         <v>46265</v>
       </c>
-      <c r="B2205" t="n">
+      <c r="B2205" s="0" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -17683,7 +17684,7 @@
       <c r="A2206" s="1" t="n">
         <v>46266</v>
       </c>
-      <c r="B2206" t="n">
+      <c r="B2206" s="0" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -17691,7 +17692,7 @@
       <c r="A2207" s="1" t="n">
         <v>46267</v>
       </c>
-      <c r="B2207" t="n">
+      <c r="B2207" s="0" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -17699,7 +17700,7 @@
       <c r="A2208" s="1" t="n">
         <v>46268</v>
       </c>
-      <c r="B2208" t="n">
+      <c r="B2208" s="0" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -17707,7 +17708,7 @@
       <c r="A2209" s="1" t="n">
         <v>46269</v>
       </c>
-      <c r="B2209" t="n">
+      <c r="B2209" s="0" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -17715,7 +17716,7 @@
       <c r="A2210" s="1" t="n">
         <v>46270</v>
       </c>
-      <c r="B2210" t="n">
+      <c r="B2210" s="0" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -17723,7 +17724,7 @@
       <c r="A2211" s="1" t="n">
         <v>46271</v>
       </c>
-      <c r="B2211" t="n">
+      <c r="B2211" s="0" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -17731,7 +17732,7 @@
       <c r="A2212" s="1" t="n">
         <v>46272</v>
       </c>
-      <c r="B2212" t="n">
+      <c r="B2212" s="0" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -17739,7 +17740,7 @@
       <c r="A2213" s="1" t="n">
         <v>46273</v>
       </c>
-      <c r="B2213" t="n">
+      <c r="B2213" s="0" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -17747,7 +17748,7 @@
       <c r="A2214" s="1" t="n">
         <v>46274</v>
       </c>
-      <c r="B2214" t="n">
+      <c r="B2214" s="0" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -17755,8 +17756,24 @@
       <c r="A2215" s="1" t="n">
         <v>46275</v>
       </c>
-      <c r="B2215" t="n">
+      <c r="B2215" s="0" t="n">
         <v>0.7</v>
+      </c>
+    </row>
+    <row r="2216">
+      <c r="A2216" s="5" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B2216" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="2217">
+      <c r="A2217" s="5" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B2217" t="n">
+        <v>0.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>